<commit_message>
Cập nhật kiểm tra ID bảng Ngọc Anh theo file Freightek mới (đã xóa 3 đơn trùng)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUdGF8bCu7bMk3Azyb5hv9
</commit_message>
<xml_diff>
--- a/09-CONG-TY-LOGISTICS-FTG/KIEM-TRA-ID-FREIGHTEK-NGOC-ANH-2026-10-20.xlsx
+++ b/09-CONG-TY-LOGISTICS-FTG/KIEM-TRA-ID-FREIGHTEK-NGOC-ANH-2026-10-20.xlsx
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nguồn: dataTable_1.xlsx (xuất Freightek) đối chiếu n.a.xlsx (bảng theo dõi), cột AI "Mã đơn web" = ID đơn. Kiểm tra ngày 20/10/2026.</t>
+          <t>Nguồn: dataTable_2.xlsx (xuất Freightek sau khi xóa đơn trùng) đối chiếu n.a.xlsx (bảng theo dõi), cột AI "Mã đơn web" = ID đơn. Kiểm tra ngày 20/10/2026.</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -549,11 +549,11 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Đơn Freightek chưa có trong Excel (đều là đơn tạo trùng)</t>
+          <t>Đơn Freightek chưa có trong Excel</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -607,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -647,322 +647,268 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Đơn trùng trên Freightek (nên hủy)</t>
+          <t>Đã xử lý</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>RLT-I2610121</t>
+          <t>RLT-I2610121, RFC-I2610120, RFC-I2609329</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Không có trong Excel</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Pending/Chờ xác nhận, chưa có xe. Trùng với RLT-I2610135 (STT 61): cùng mã IFTZ-ZBL-260923046, cùng ngày 29/9–1/10, cùng tuyến Tiên Sơn → An Phước Đồng Nai, tạo cùng ngày 05/10.</t>
+          <t>Ba đơn tạo trùng đã được xóa khỏi Freightek (không còn trong file xuất dataTable_2).</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Xác nhận là đơn tạo trùng rồi hủy/xóa trên Freightek.</t>
+          <t>Xong.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Đơn trùng trên Freightek (nên hủy)</t>
+          <t>Đã xử lý</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>RFC-I2610120</t>
+          <t>RFT-I2609660</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Không có trong Excel</t>
+          <t>STT 60 (dòng 79)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Pending/Chờ xác nhận, chưa có xe. Trùng với RFC-I2610128 (STT 63): cùng khách Hưng Giang, cùng ngày 30/9–1/10, cùng tuyến Tân Thanh → Lương Sơn, tạo cùng ngày 05/10.</t>
+          <t>Đơn đã có trên Freightek: xe 12H 05295, 28/9–29/9, Hữu Nghị → Tiên Sơn, lợi nhuận 3,95 USD (≈ 103.500đ, khớp Excel). Ô Trucking No. đang ghi lặp "12H 05295; 12H 05295".</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Xác nhận là đơn tạo trùng rồi hủy/xóa trên Freightek.</t>
+          <t>Khớp. Có thể sửa Trucking No. còn 1 biển.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Đơn trùng trên Freightek (nên hủy)</t>
+          <t>Thiếu ID</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>RFC-I2609329</t>
+          <t>(chưa có ID)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Không có trong Excel</t>
+          <t>STT 62 (dòng 81)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Pending/Chờ xác nhận. Ghi chú giống hệt RFC-I2609330 (STT 45): R73196, lái xe Nguyễn Tiến Dũng, xe 98H04455, cùng ngày 10/9–11/9.</t>
+          <t>TM, xe 98E01083 (C&amp;T), Hữu Nghị → Tiên Sơn, 26/8, ghi chú "về kho, đơn t8". Chi phí NCC 2.352.000, chưa có doanh thu KH. File Freightek chỉ có đơn tháng 9 nên chưa đối chiếu được.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Xác nhận là đơn tạo trùng rồi hủy/xóa trên Freightek.</t>
+          <t>Kiểm tra đơn tháng 8 trên Freightek rồi điền ID.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Cần kiểm tra trên Freightek</t>
+          <t>Lệch ngày + biển số</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>RFT-I2609660</t>
+          <t>RFT-I2609377</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>STT 60 (dòng 79)</t>
+          <t>STT 41 (dòng 52)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>TM, xe 12H 05295 (Hoàng Văn Nho), Hữu Nghị → Tiên Sơn, 28/9–29/9, đã xuất HĐ NCC số 817. ID này không có trong file xuất Freightek, và không đơn nào mang biển 12H05295.</t>
+          <t>Excel: ngày 16/9. Freightek: ETD 9/9, ETA 10/9. Ngoài ra cột BKS (cả Excel và Freightek) ghi 29E75450 nhưng thông tin xe lại là "biển vàng 30M-896.82, Lưu Quyết Thắng". 29E75450 là xe của đơn RFT-I2609735 (STT 38) cùng ngày 16/9.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Tìm ID trên Freightek; nếu sai ID thì sửa, nếu chưa có thì tạo đơn.</t>
+          <t>Xác định ngày chạy và xe thật, sửa cho thống nhất ở cả hai nơi.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Thiếu ID</t>
+          <t>Lệch ngày</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>(chưa có ID)</t>
+          <t>RLT-E2609652</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>STT 62 (dòng 81)</t>
+          <t>STT 53 (dòng 71)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>TM, xe 98E01083 (C&amp;T), Hữu Nghị → Tiên Sơn, 26/8, ghi chú "về kho, đơn t8". Chi phí NCC 2.352.000, chưa có doanh thu KH. File Freightek chỉ có đơn tháng 9 nên chưa đối chiếu được.</t>
+          <t>Excel: lấy 24/9, giao 28/9. Freightek: ETD 28/9, ETA 29/9.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Kiểm tra đơn tháng 8 trên Freightek rồi điền ID.</t>
+          <t>Thống nhất ngày lấy/giao.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Lệch ngày + biển số</t>
+          <t>Cần sửa trên Freightek</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>RFT-I2609377</t>
+          <t>RFC-E2609742</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>STT 41 (dòng 52)</t>
+          <t>STT 64 (dòng 83)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Excel: ngày 16/9. Freightek: ETD 9/9, ETA 10/9. Ngoài ra cột BKS (cả Excel và Freightek) ghi 29E75450 nhưng thông tin xe lại là "biển vàng 30M-896.82, Lưu Quyết Thắng". 29E75450 là xe của đơn RFT-I2609735 (STT 38) cùng ngày 16/9.</t>
+          <t>ETA trên Freightek là 28/10/2026, Excel giao 28/9/2026.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Xác định ngày chạy và xe thật, sửa cho thống nhất ở cả hai nơi.</t>
+          <t>Nhiều khả năng gõ nhầm tháng → sửa ETA thành 28/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Lệch ngày</t>
+          <t>Cần cập nhật trạng thái</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>RLT-E2609652</t>
+          <t>RFT-I2609725, RFT-I2609736, RFC-I2609649, RFC-D2609638</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>STT 53 (dòng 71)</t>
+          <t>STT 24, 42, 52, 57</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Excel: lấy 24/9, giao 28/9. Freightek: ETD 28/9, ETA 29/9.</t>
+          <t>Chuyến đã chạy trong tháng 9 nhưng trên Freightek vẫn "Chờ xác nhận" / Pending.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Thống nhất ngày lấy/giao.</t>
+          <t>Xác nhận đơn trên Freightek.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cần sửa trên Freightek</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>RFC-E2609742</t>
+          <t>RFT-I2609282, RFT-I2609735</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>STT 64 (dòng 83)</t>
+          <t>STT 32, 38</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>ETA trên Freightek là 28/10/2026, Excel giao 28/9/2026.</t>
+          <t>Ô "Mã đơn web" chứa 2 mã: "FTG2609157 / RFT-I2609282" và "FTG2609166 / RFT-I2609735". Mã RFT khớp Freightek.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Nhiều khả năng gõ nhầm tháng → sửa ETA thành 28/09/2026.</t>
+          <t>Nên để riêng mã FTG ra cột khác để lọc theo ID không bị lỗi.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Cần cập nhật trạng thái</t>
+          <t>Ghi chú</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>RFT-I2609725, RFT-I2609736, RFC-I2609649, RFC-D2609638</t>
+          <t>RFT-I2609153</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>STT 24, 42, 52, 57</t>
+          <t>STT 44 (dòng 62)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Chuyến đã chạy trong tháng 9 nhưng trên Freightek vẫn "Chờ xác nhận" / Pending.</t>
+          <t>Dòng chi phí lưu ca + vé bãi 650.000; cột BKS trong Excel để trống (thông tin xe là 12H04341, khớp Freightek).</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Xác nhận đơn trên Freightek.</t>
+          <t>Điền 12H04341 vào cột BKS.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Ghi chú</t>
+          <t>Không cần xử lý</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>RFT-I2609282, RFT-I2609735</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>STT 32, 38</t>
+          <t>15 dòng không có STT</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Ô "Mã đơn web" chứa 2 mã: "FTG2609157 / RFT-I2609282" và "FTG2609166 / RFT-I2609735". Mã RFT khớp Freightek.</t>
+          <t>Các dòng không STT (dòng 13, 20, 29, 31, 36, 38, 49, 55–61, 74) là các lô hàng IFTZ-ZBL ghép chung xe với chuyến ngay phía trên, chỉ có cước thu KH.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Nên để riêng mã FTG ra cột khác để lọc theo ID không bị lỗi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>RFT-I2609153</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>STT 44 (dòng 62)</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Dòng chi phí lưu ca + vé bãi 650.000; cột BKS trong Excel để trống (thông tin xe là 12H04341, khớp Freightek).</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Điền 12H04341 vào cột BKS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Không cần xử lý</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>15 dòng không có STT</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>Các dòng không STT (dòng 13, 20, 29, 31, 36, 38, 49, 55–61, 74) là các lô hàng IFTZ-ZBL ghép chung xe với chuyến ngay phía trên, chỉ có cước thu KH.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Thuộc đơn của dòng có STT ngay phía trên, không cần ID riêng.</t>
         </is>
@@ -4929,14 +4875,30 @@
           <t>RFT-I2609660</t>
         </is>
       </c>
-      <c r="J61" s="3" t="n"/>
-      <c r="K61" s="3" t="n"/>
-      <c r="L61" s="3" t="n"/>
-      <c r="M61" s="3" t="n"/>
-      <c r="N61" s="3" t="n"/>
-      <c r="O61" s="6" t="inlineStr">
-        <is>
-          <t>ID không có trên Freightek</t>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Tongmao</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>12H 05295; 12H 05295</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M61" s="4" t="n">
+        <v>46294</v>
+      </c>
+      <c r="N61" s="3" t="inlineStr">
+        <is>
+          <t>Xe đến điểm giao hàng / Active</t>
+        </is>
+      </c>
+      <c r="O61" s="3" t="inlineStr">
+        <is>
+          <t>Khớp</t>
         </is>
       </c>
     </row>

</xml_diff>